<commit_message>
with programmable readout timeout and fixed bug for event FULL_SIZE
Added programmable EVENT_TIMEOUT via register 6 and fixed field length of FULL_SIZE in DigiInterface/ROCFifoController
</commit_message>
<xml_diff>
--- a/DRAC_Registers_timingconstrained.xlsx
+++ b/DRAC_Registers_timingconstrained.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tecchio/Desktop/work_instructions/ROC Manuals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72094A9E-104F-3B4D-A69C-E6F801196C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE21BBA-36A2-BD46-BB7D-EB7020B6E4D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1400" yWindow="760" windowWidth="20140" windowHeight="18020" xr2:uid="{8033228E-8299-4C41-92C5-FE54786B42FA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="256">
   <si>
     <t>address</t>
   </si>
@@ -227,18 +227,6 @@
     <t xml:space="preserve">    Serdes DIGI FIFO  EMPTY status</t>
   </si>
   <si>
-    <t>DREQ FIFO RD status 1st</t>
-  </si>
-  <si>
-    <t>DREQ FIFO WR status 1st</t>
-  </si>
-  <si>
-    <t>DREQ FIFO WR status end</t>
-  </si>
-  <si>
-    <t>DREQ FIFO RD status end</t>
-  </si>
-  <si>
     <t>27&amp;28</t>
   </si>
   <si>
@@ -260,9 +248,6 @@
     <t>33&amp;34</t>
   </si>
   <si>
-    <t>counter of Data Request packets from DTC : 9=&gt;bit(15:0), 10=&gt;bit(31:16)</t>
-  </si>
-  <si>
     <t>counter of Event Markers from DTC: 11=&gt;bit(15:0), 12=&gt;bit(31:16)</t>
   </si>
   <si>
@@ -272,9 +257,6 @@
     <t>counter of NULL Heartbeat packets from DTC : 29=&gt;bit(15:0), 30=&gt;bit(31:16)</t>
   </si>
   <si>
-    <t>counter TAG written to DDR minus number of TAG read from DDR : 31=&gt;bit(15:0), 32=&gt;bit(31:16)32</t>
-  </si>
-  <si>
     <t>DCS_PREFCNT</t>
   </si>
   <si>
@@ -311,18 +293,6 @@
     <t>counter PREFETCH packets from DTC  : 33=&gt;bit(15:0), 34=&gt;bit(31:16)</t>
   </si>
   <si>
-    <t>counter tags written by DDR  : 35=&gt;bit(15:0), 36=&gt;bit(31:16)</t>
-  </si>
-  <si>
-    <t>counter tags read frm DDR: 37=&gt;bit(15:0), 38=&gt;bit(31:16)</t>
-  </si>
-  <si>
-    <t>counter tags sent to DTC: 38=&gt;bit(15:0), 39=&gt;bit(31:16)</t>
-  </si>
-  <si>
-    <t>counter tags sent to DTC with null data: 41=&gt;bit(15:0), 42=&gt;bit(31:16)</t>
-  </si>
-  <si>
     <t>45&amp;46&amp;47</t>
   </si>
   <si>
@@ -353,21 +323,6 @@
     <t>DCS_OFFSETTAG</t>
   </si>
   <si>
-    <t>tag of first HB in a new spill 57=&gt;bit(15:0), 58=&gt;bit(31:16), 59=&gt;bit(47:32)</t>
-  </si>
-  <si>
-    <t>tag of last Heartbeat packet from DTC: 45=&gt;bit(15:0), 46=&gt;bit(31:16), 47=&gt;bit(47:32)</t>
-  </si>
-  <si>
-    <t>tag of last Prefetch packet from DTC: 48=&gt;bit(15:0), 49=&gt;bit(31:16), 50=&gt;bit(47:32)</t>
-  </si>
-  <si>
-    <t>tag of last Prefetch OR DREQ packet from DTC: 51=&gt;bit(15:0), 52=&gt;bit(31:16), 53=&gt;bit(47:32)</t>
-  </si>
-  <si>
-    <t>tag of last Data Request packet from DTC: 54=&gt;bit(15:0), 55=&gt;bit(31:16), 56=&gt;bit(47:32)</t>
-  </si>
-  <si>
     <t xml:space="preserve">    DCS_FORCE_FULL</t>
   </si>
   <si>
@@ -392,18 +347,12 @@
     <t>DCS_EVMCNT</t>
   </si>
   <si>
-    <t>counter of event windows seen : 64=&gt;bit(15:0), 65=&gt;bit(31:16)</t>
-  </si>
-  <si>
     <t>66&amp;67&amp;68</t>
   </si>
   <si>
     <t>DCS_FULLTAG</t>
   </si>
   <si>
-    <t>tag of first TAG for which DREQ is full 66=&gt;bit(15:0), 67=&gt;bit(31:16), 68=&gt;bit(47:32)</t>
-  </si>
-  <si>
     <t>TWI BUSY status</t>
   </si>
   <si>
@@ -485,27 +434,15 @@
     <t>0=TRK, 1=CAL, 2-CRV, 4=STM, 5=EXTMON</t>
   </si>
   <si>
-    <t>(*) error 1 =&gt; event tag to DDR, 2=&gt; event size, 3=&gt; event block size, 4=&gt; event error or overflow, 5=&gt;event tag from DDR</t>
-  </si>
-  <si>
     <t>First version: Aug 13, 2024</t>
   </si>
   <si>
-    <t>Last updated: Nov 17, 2024</t>
-  </si>
-  <si>
     <t>(7:4)</t>
   </si>
   <si>
     <t>(11:8)</t>
   </si>
   <si>
-    <t>bit(8)-&gt; CAL lane 0;  (9)-&gt;CAL lane 1; (10)-&gt;HV lane 0; (11) -&gt; HV lane 1</t>
-  </si>
-  <si>
-    <t>bit(4)-&gt; CAL lane 0;  (5)-&gt;CAL lane 1;  (6)-&gt;HV lane 0;   (7) -&gt; HV lane 1</t>
-  </si>
-  <si>
     <t>(10:0)</t>
   </si>
   <si>
@@ -527,30 +464,12 @@
     <t>unused bit(7:3) &amp; (11:10) &amp; (15:13) tied to zero</t>
   </si>
   <si>
-    <t>bit(3:0)=MSB of counter data to DREQ_FIFO,  bit(9:8)=STORE_POS(**); bit(12)=DREQ_FIFO FULL status</t>
-  </si>
-  <si>
-    <t>bit(3:0)=MSB of counter read from DREQ FIFO; bit(9:8)=FETCH_POS (**); bit(12)=DREQ_FIFO EMPTYstatus</t>
-  </si>
-  <si>
-    <t>LSB of counter of 40-bit data stored to DREQ_FIFO</t>
-  </si>
-  <si>
-    <t>LSB of counter of 40-bit data fetched from DREQ_FIFO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(**) DREQ_FIFO 40-bit contain the size(***) from 3 consecutive tags in bit(12:0),(25:13) and (38:26), respectively. STORE_POS and FETCH_POS are 0,1 and 2 for the 3 possible tags. </t>
-  </si>
-  <si>
     <t xml:space="preserve">(***) The 13 bits for each tag contain: bit(9:0) event size in number of hits, bit(10) = event size overflow (ie if more than 255 hits), bit(11) = event with tag sync (^), bit(12) DDR wraparound event </t>
   </si>
   <si>
     <t>(^) Tag sync error is the OR of DIGI synchronization error and inconsistent tags among SERDES. A synchronization signal is sent by the ROC to the DIGIS every 16384 event windows. If DIGI local window tag counter does not agree, tag sync error is pulled is set by the DIGI</t>
   </si>
   <si>
-    <t>local event tag counter sent by DIGI to ROC</t>
-  </si>
-  <si>
     <t>bit(0) for CAL_DGI TWI;  bit(4) for HV_DIGI TWI</t>
   </si>
   <si>
@@ -602,9 +521,6 @@
     <t>(31:0)</t>
   </si>
   <si>
-    <t>(63:0)</t>
-  </si>
-  <si>
     <t>DCS_to_SERIAL</t>
   </si>
   <si>
@@ -626,21 +542,9 @@
     <t>Can also be set by serial address 0x17 (23)</t>
   </si>
   <si>
-    <t>(15:12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Unused</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Lane_empty_seen</t>
   </si>
   <si>
-    <t>set to 0x0</t>
-  </si>
-  <si>
-    <t>Set to 1 at first EMPTY falling edge, set to 0 after EW_DONE</t>
-  </si>
-  <si>
     <t>number of EW_DONE to EW_FIFO_Controller</t>
   </si>
   <si>
@@ -701,9 +605,6 @@
     <t>TWI ADDR to HV DIGI(*)</t>
   </si>
   <si>
-    <t>(*) Enabled by DCS_DIGIRW_SEL via adrr. 6</t>
-  </si>
-  <si>
     <t>DCS_MEM_READ</t>
   </si>
   <si>
@@ -728,24 +629,12 @@
     <t>Read data recorded in error counter passed by addr=17  (unused)</t>
   </si>
   <si>
-    <t>Read status bit below:</t>
-  </si>
-  <si>
-    <t>bit(0)-&gt; CAL lane 0;  (1)-&gt;CAL lane 1;  (2)-&gt;HV lane 0;   (3) -&gt; HV lane 1</t>
-  </si>
-  <si>
     <t>DDR dump FIFO WR status</t>
   </si>
   <si>
     <t>DDR dump FIFO RD status</t>
   </si>
   <si>
-    <t>bit(15)=FIFO FULL, bit(7:0) =FIFO WRCNT</t>
-  </si>
-  <si>
-    <t>bit(15)=FIFO EMPTY, bit(9:0) =FIFO RDCNT</t>
-  </si>
-  <si>
     <t>DDR dump FIFO is 64 bit IN and 16 bit out, hence different number of WR_COUNT vs RD_COUNT words</t>
   </si>
   <si>
@@ -773,29 +662,155 @@
     <t>(15; 4:0)</t>
   </si>
   <si>
-    <t>bit(15:0) of start address, in units of 1KB, of last DDR read</t>
-  </si>
-  <si>
-    <t>DCS_DDR_ADDRESS LSB</t>
-  </si>
-  <si>
-    <t>DCS_DDR_ADDRESS MSB</t>
-  </si>
-  <si>
-    <t>bit(19:16) of start address, in units of 1KB, of last DDR read</t>
-  </si>
-  <si>
     <t>DCS_DIAG_DATA</t>
   </si>
   <si>
-    <t xml:space="preserve">Number of payload 160bit words in uProc command via fiber </t>
+    <t>15&amp;16</t>
+  </si>
+  <si>
+    <t>DCS_DDR_ADDRESS</t>
+  </si>
+  <si>
+    <t>counter of Data Request packets from DTC: 9=&gt;bit(15:0), 10=&gt;bit(31:16)</t>
+  </si>
+  <si>
+    <t>DDR address of last read, in units of 1KB: 15=&gt;bit(15:0), 16=&gt;bit(19:16)</t>
+  </si>
+  <si>
+    <t>(19:0)</t>
+  </si>
+  <si>
+    <t>DREQ FIFO WRCNT (LSB)</t>
+  </si>
+  <si>
+    <t>DREQ FIFO WR status</t>
+  </si>
+  <si>
+    <t>bit(3:0)=DREQ_FIFO_WRCNT(19:0),  bit(9:8)=STORE_POS(**); bit(12)=DREQ_FIFO FULL status</t>
+  </si>
+  <si>
+    <t>Set to 1 at first EMPTY falling edge, set to 0 after full serdes is read</t>
+  </si>
+  <si>
+    <t>bit(15:0) of counter of 40-bit data stored to DREQ_FIFO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(**) DREQ_FIFO 40-bit contain the event size(***) from 3 consecutive tags in bit(12:0),(25:13) and (38:26), respectively. STORE_POS and FETCH_POS are 0,1 and 2 for the 3 possible tags. </t>
+  </si>
+  <si>
+    <t>DREQ FIFO RDCNT (LSB)</t>
+  </si>
+  <si>
+    <t>bit(15:0) of counter of 40-bit data fetched from DREQ_FIFO</t>
+  </si>
+  <si>
+    <t>bit(15)=FIFO EMPTY, bit(9:0) =FIFO RDCNT (in units of 16-bit words)</t>
+  </si>
+  <si>
+    <t>bit(3:0)=DREQ_FIFO_RDCNT(19:0); bit(9:8)=FETCH_POS (**); bit(12)=DREQ_FIFO EMPTYstatus</t>
+  </si>
+  <si>
+    <t>(11:0)</t>
+  </si>
+  <si>
+    <t>(12:0)</t>
+  </si>
+  <si>
+    <t>Read status bit as listed below:</t>
+  </si>
+  <si>
+    <t>DREQ FIFO RD status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      bit(0)-&gt; CAL lane 0;  (1)-&gt;CAL lane 1;  (2)-&gt;HV lane 0;   (3) -&gt; HV lane 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      bit(4)-&gt; CAL lane 0;  (5)-&gt;CAL lane 1;  (6)-&gt;HV lane 0;   (7) -&gt; HV lane 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      bit(8)-&gt; CAL lane 0;  (9)-&gt;CAL lane 1; (10)-&gt;HV lane 0; (11) -&gt; HV lane 1</t>
+  </si>
+  <si>
+    <t>bit(15)=FIFO FULL, bit(7:0) =FIFO WRCNT (in units of 64-bit words)</t>
+  </si>
+  <si>
+    <t>counter of EVENTS written by DDR  : 35=&gt;bit(15:0), 36=&gt;bit(31:16)</t>
+  </si>
+  <si>
+    <t>counter of EVENTS read from DDR: 37=&gt;bit(15:0), 38=&gt;bit(31:16)</t>
+  </si>
+  <si>
+    <t>counter of EVM sent by DTC minus number of EVENTS written to  DDR : 31=&gt;bit(15:0), 32=&gt;bit(31:16)</t>
+  </si>
+  <si>
+    <t>counter of EVENTS sent to DTC: 38=&gt;bit(15:0), 39=&gt;bit(31:16)</t>
+  </si>
+  <si>
+    <t>counter of EVENTS sent to DTC with null data: 41=&gt;bit(15:0), 42=&gt;bit(31:16)</t>
+  </si>
+  <si>
+    <t>local counter of EVENTS sent by DIGI to ROC (reset to zero after a null HB)</t>
+  </si>
+  <si>
+    <t>TAG of last Heartbeat packet from DTC: 45=&gt;bit(15:0), 46=&gt;bit(31:16), 47=&gt;bit(47:32)</t>
+  </si>
+  <si>
+    <t>TAG of last Prefetch packet from DTC: 48=&gt;bit(15:0), 49=&gt;bit(31:16), 50=&gt;bit(47:32)</t>
+  </si>
+  <si>
+    <t>TAG of last Prefetch OR DREQ packet from DTC: 51=&gt;bit(15:0), 52=&gt;bit(31:16), 53=&gt;bit(47:32)</t>
+  </si>
+  <si>
+    <t>TAG of last Data Request packet from DTC: 54=&gt;bit(15:0), 55=&gt;bit(31:16), 56=&gt;bit(47:32)</t>
+  </si>
+  <si>
+    <t>TAG of first HB in a new spill 57=&gt;bit(15:0), 58=&gt;bit(31:16), 59=&gt;bit(47:32)</t>
+  </si>
+  <si>
+    <t>counter of EVENT WINDOWS seen : 64=&gt;bit(15:0), 65=&gt;bit(31:16)</t>
+  </si>
+  <si>
+    <t>TAG of first TAG for which DREQ is full 66=&gt;bit(15:0), 67=&gt;bit(31:16), 68=&gt;bit(47:32)</t>
+  </si>
+  <si>
+    <t>60&amp;61</t>
+  </si>
+  <si>
+    <t>EVENT_TIMEOUT</t>
+  </si>
+  <si>
+    <t>Maximum time allowed from DATA REQUEST to event in DDR ready to be read: 15=&gt;bit(15:0), 16=&gt;bit(19:16)</t>
+  </si>
+  <si>
+    <t>In units of 12.5 ns</t>
+  </si>
+  <si>
+    <t>(14:0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of payload 16-bit words in uProc command via fiber </t>
+  </si>
+  <si>
+    <t>Read data recorded in error counter passed by addr=17</t>
+  </si>
+  <si>
+    <t>0xFFFF</t>
+  </si>
+  <si>
+    <t>(*) Enabled by DCS_DIGIRW_SEL via reg=6</t>
+  </si>
+  <si>
+    <t>Last updated: May 4, 2025</t>
+  </si>
+  <si>
+    <t>in units of 12.5 ns (80 MHz clock)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -845,6 +860,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="6"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -866,7 +888,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -895,6 +917,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1209,23 +1235,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{518204DB-35D9-1947-A6E3-732720EF0C47}">
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.1640625" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.1640625" customWidth="1"/>
-    <col min="3" max="3" width="63.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="91" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.1640625" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -1258,19 +1284,19 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>239</v>
+        <v>202</v>
       </c>
       <c r="C6" t="s">
-        <v>242</v>
+        <v>205</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>240</v>
+        <v>203</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>241</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -1284,7 +1310,7 @@
         <v>28</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1295,16 +1321,16 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>189</v>
+        <v>161</v>
       </c>
       <c r="C8" t="s">
-        <v>191</v>
+        <v>163</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="E8" t="s">
-        <v>190</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -1312,10 +1338,10 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>192</v>
+        <v>164</v>
       </c>
       <c r="C9" t="s">
-        <v>203</v>
+        <v>171</v>
       </c>
       <c r="D9" s="6">
         <v>0</v>
@@ -1335,7 +1361,7 @@
         <v>29</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="E10" t="s">
         <v>3</v>
@@ -1349,7 +1375,7 @@
         <v>30</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -1427,13 +1453,13 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B17" s="10" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="C17" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -1455,10 +1481,10 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B19" s="10" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="C19" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>41</v>
@@ -1472,10 +1498,10 @@
         <v>9</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="C20" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
       <c r="D20" s="6">
         <v>0</v>
@@ -1484,7 +1510,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="s">
-        <v>195</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -1495,7 +1521,7 @@
         <v>43</v>
       </c>
       <c r="C21" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="D21" s="6">
         <v>0</v>
@@ -1504,7 +1530,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -1515,7 +1541,7 @@
         <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>44</v>
@@ -1524,135 +1550,132 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="6">
-        <v>23</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="C23" t="s">
-        <v>209</v>
-      </c>
-      <c r="D23" s="6">
-        <v>0</v>
-      </c>
-      <c r="E23">
-        <v>0</v>
-      </c>
-      <c r="F23" t="s">
-        <v>45</v>
+        <v>176</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="14">
+        <v>17</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>216</v>
+        <v>183</v>
       </c>
       <c r="C24" t="s">
-        <v>210</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>161</v>
+        <v>177</v>
+      </c>
+      <c r="D24" s="6">
+        <v>0</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
       <c r="F24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="6">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>217</v>
+        <v>184</v>
       </c>
       <c r="C25" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="E25">
         <v>0</v>
+      </c>
+      <c r="F25" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>218</v>
+        <v>185</v>
       </c>
       <c r="C26" t="s">
-        <v>212</v>
-      </c>
-      <c r="D26" s="6">
-        <v>0</v>
+        <v>179</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>136</v>
       </c>
       <c r="E26">
         <v>0</v>
-      </c>
-      <c r="F26" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>219</v>
+        <v>186</v>
       </c>
       <c r="C27" t="s">
-        <v>213</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>161</v>
+        <v>180</v>
+      </c>
+      <c r="D27" s="6">
+        <v>0</v>
       </c>
       <c r="E27">
         <v>0</v>
       </c>
       <c r="F27" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>220</v>
+        <v>187</v>
       </c>
       <c r="C28" t="s">
-        <v>214</v>
+        <v>181</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="E28">
         <v>0</v>
+      </c>
+      <c r="F28" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="6">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>47</v>
+        <v>188</v>
       </c>
       <c r="C29" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -1660,153 +1683,156 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="6">
+        <v>29</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" t="s">
+        <v>127</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" s="6">
         <v>30</v>
       </c>
-      <c r="B30" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="C30" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="E30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31" s="11">
-        <v>31</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="D31" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="E31" s="4">
-        <v>0</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>148</v>
+      <c r="B31" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C31" t="s">
+        <v>128</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="11">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>222</v>
+        <v>129</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="D32" s="11">
-        <v>0</v>
+        <v>130</v>
+      </c>
+      <c r="D32" s="11" t="s">
+        <v>139</v>
       </c>
       <c r="E32" s="4">
         <v>0</v>
       </c>
-      <c r="F32" s="4"/>
+      <c r="F32" s="4" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="11">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>224</v>
+        <v>189</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="D33" s="11" t="s">
-        <v>157</v>
+        <v>190</v>
+      </c>
+      <c r="D33" s="11">
+        <v>0</v>
       </c>
       <c r="E33" s="4">
         <v>0</v>
       </c>
-      <c r="F33" s="4" t="s">
-        <v>226</v>
-      </c>
+      <c r="F33" s="4"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="11">
+        <v>33</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="E34" s="4">
+        <v>0</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" s="11">
         <v>34</v>
       </c>
-      <c r="B34" s="12" t="s">
-        <v>225</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="D34" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="E34" s="4">
-        <v>0</v>
-      </c>
-      <c r="F34" s="4"/>
+      <c r="B35" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="E35" s="4">
+        <v>0</v>
+      </c>
+      <c r="F35" s="4"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B36" s="10" t="s">
-        <v>221</v>
+      <c r="A36" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="D36" s="11" t="s">
+        <v>213</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="10" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B40" s="5" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A39" s="6">
-        <v>0</v>
-      </c>
-      <c r="B39" t="s">
-        <v>5</v>
-      </c>
-      <c r="C39" t="s">
-        <v>48</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="E39" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A40" s="6">
-        <v>1</v>
-      </c>
-      <c r="B40" t="s">
-        <v>239</v>
-      </c>
-      <c r="C40" t="s">
-        <v>243</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="E40" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B41" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C41" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>157</v>
+        <v>48</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>136</v>
       </c>
       <c r="E41" t="s">
         <v>3</v>
@@ -1814,16 +1840,16 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B42" t="s">
-        <v>8</v>
+        <v>202</v>
       </c>
       <c r="C42" t="s">
-        <v>9</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>157</v>
+        <v>206</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>207</v>
       </c>
       <c r="E42" t="s">
         <v>3</v>
@@ -1831,16 +1857,16 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B43" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C43" t="s">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="E43" t="s">
         <v>3</v>
@@ -1848,33 +1874,33 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>189</v>
+        <v>8</v>
       </c>
       <c r="C44" t="s">
-        <v>193</v>
+        <v>9</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="F44" t="s">
-        <v>194</v>
+        <v>136</v>
+      </c>
+      <c r="E44" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B45" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>50</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>157</v>
+        <v>49</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>135</v>
       </c>
       <c r="E45" t="s">
         <v>3</v>
@@ -1882,863 +1908,893 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B46" t="s">
-        <v>12</v>
+        <v>161</v>
       </c>
       <c r="C46" t="s">
-        <v>13</v>
-      </c>
-      <c r="D46" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="E46" t="s">
-        <v>3</v>
+        <v>165</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="F46" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="C47" t="s">
-        <v>114</v>
+        <v>50</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="E47" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A48" s="6" t="s">
+      <c r="A48" s="6">
+        <v>7</v>
+      </c>
+      <c r="B48" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" t="s">
+        <v>13</v>
+      </c>
+      <c r="D48" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="E48" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A49" s="6">
+        <v>8</v>
+      </c>
+      <c r="B49" t="s">
+        <v>53</v>
+      </c>
+      <c r="C49" t="s">
+        <v>99</v>
+      </c>
+      <c r="D49" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="E49" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A50" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B50" t="s">
         <v>54</v>
       </c>
-      <c r="C48" t="s">
-        <v>74</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="F48" s="3"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A49" s="6" t="s">
+      <c r="C50" t="s">
+        <v>211</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="F50" s="3"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A51" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B51" t="s">
         <v>56</v>
       </c>
-      <c r="C49" t="s">
-        <v>75</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="F49" s="2"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A50" s="6">
-        <v>13</v>
-      </c>
-      <c r="B50" t="s">
-        <v>57</v>
-      </c>
-      <c r="C50" t="s">
-        <v>58</v>
-      </c>
-      <c r="D50" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="F50" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A51" s="6">
-        <v>14</v>
-      </c>
-      <c r="B51" t="s">
-        <v>202</v>
-      </c>
       <c r="C51" t="s">
-        <v>201</v>
-      </c>
-      <c r="D51" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="F51" t="s">
-        <v>115</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="F51" s="2"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="6">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B52" t="s">
-        <v>246</v>
+        <v>57</v>
       </c>
       <c r="C52" t="s">
-        <v>245</v>
+        <v>58</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>157</v>
+        <v>136</v>
+      </c>
+      <c r="F52" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="6">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B53" t="s">
-        <v>247</v>
+        <v>170</v>
       </c>
       <c r="C53" t="s">
-        <v>248</v>
+        <v>169</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>158</v>
+        <v>136</v>
+      </c>
+      <c r="F53" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A54" s="6">
+      <c r="A54" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B54" t="s">
+        <v>210</v>
+      </c>
+      <c r="C54" t="s">
+        <v>212</v>
+      </c>
+      <c r="D54" s="11" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A55" s="14">
         <v>17</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B55" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="C54" t="s">
-        <v>229</v>
-      </c>
-      <c r="D54" s="6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A55" s="6">
+      <c r="C55" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A56" s="6">
         <v>18</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B56" t="s">
         <v>60</v>
       </c>
-      <c r="C55" t="s">
-        <v>230</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B56" t="s">
-        <v>198</v>
-      </c>
       <c r="C56" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="F56" t="s">
-        <v>200</v>
+        <v>224</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
-        <v>61</v>
+        <v>168</v>
       </c>
       <c r="C57" t="s">
-        <v>155</v>
+        <v>228</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>152</v>
+        <v>137</v>
+      </c>
+      <c r="F57" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C58" t="s">
-        <v>154</v>
+        <v>229</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>153</v>
+        <v>133</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
-        <v>197</v>
+        <v>62</v>
       </c>
       <c r="C59" t="s">
-        <v>199</v>
+        <v>230</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A60" s="6">
-        <v>20</v>
-      </c>
-      <c r="B60" t="s">
-        <v>232</v>
-      </c>
-      <c r="C60" t="s">
-        <v>234</v>
-      </c>
-      <c r="D60" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="F60" t="s">
-        <v>236</v>
+        <v>134</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="6">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B61" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="C61" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>188</v>
+        <v>136</v>
+      </c>
+      <c r="F61" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="6">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B62" t="s">
-        <v>64</v>
+        <v>198</v>
       </c>
       <c r="C62" t="s">
-        <v>165</v>
-      </c>
-      <c r="D62" s="11" t="s">
-        <v>157</v>
+        <v>222</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="6">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B63" t="s">
-        <v>65</v>
+        <v>214</v>
       </c>
       <c r="C63" t="s">
-        <v>163</v>
+        <v>218</v>
       </c>
       <c r="D63" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="F63" t="s">
-        <v>162</v>
+        <v>136</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="6">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B64" t="s">
-        <v>63</v>
+        <v>215</v>
       </c>
       <c r="C64" t="s">
-        <v>166</v>
+        <v>216</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>157</v>
+        <v>225</v>
+      </c>
+      <c r="F64" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="6">
+        <v>25</v>
+      </c>
+      <c r="B65" t="s">
+        <v>220</v>
+      </c>
+      <c r="C65" t="s">
+        <v>221</v>
+      </c>
+      <c r="D65" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A66" s="6">
         <v>26</v>
       </c>
-      <c r="B65" t="s">
-        <v>66</v>
-      </c>
-      <c r="C65" t="s">
-        <v>164</v>
-      </c>
-      <c r="D65" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="F65" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A66" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B66" s="13" t="s">
-        <v>68</v>
+      <c r="B66" t="s">
+        <v>227</v>
       </c>
       <c r="C66" t="s">
-        <v>76</v>
-      </c>
-      <c r="D66" s="6" t="s">
-        <v>187</v>
+        <v>223</v>
+      </c>
+      <c r="D66" s="11" t="s">
+        <v>225</v>
       </c>
       <c r="F66" t="s">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C67" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="F67" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="6" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B68" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C68" t="s">
         <v>72</v>
       </c>
-      <c r="C68" t="s">
-        <v>78</v>
-      </c>
       <c r="D68" s="6" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="F68" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="6" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="C69" t="s">
-        <v>90</v>
+        <v>234</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="F69" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="C70" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="F70" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A71" s="11" t="s">
-        <v>81</v>
+      <c r="A71" s="6" t="s">
+        <v>74</v>
       </c>
       <c r="B71" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D71" s="11" t="s">
-        <v>187</v>
-      </c>
-      <c r="E71" s="4"/>
-      <c r="F71" s="4" t="s">
-        <v>115</v>
+        <v>76</v>
+      </c>
+      <c r="C71" t="s">
+        <v>232</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="F71" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="11" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>93</v>
+        <v>233</v>
       </c>
       <c r="D72" s="11" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="E72" s="4"/>
       <c r="F72" s="4" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="11" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="B73" s="13" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>94</v>
+        <v>235</v>
       </c>
       <c r="D73" s="11" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="E73" s="4"/>
       <c r="F73" s="4" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="11" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="B74" s="13" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>170</v>
+        <v>236</v>
       </c>
       <c r="D74" s="11" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="E74" s="4"/>
       <c r="F74" s="4" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="11" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B75" s="13" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>106</v>
+        <v>237</v>
       </c>
       <c r="D75" s="11" t="s">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="E75" s="4"/>
-      <c r="F75" s="4"/>
+      <c r="F75" s="4" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="11" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>107</v>
+        <v>238</v>
       </c>
       <c r="D76" s="11" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="E76" s="4"/>
       <c r="F76" s="4"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="11" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>108</v>
+        <v>239</v>
       </c>
       <c r="D77" s="11" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="E77" s="4"/>
       <c r="F77" s="4"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="11" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>109</v>
+        <v>240</v>
       </c>
       <c r="D78" s="11" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="E78" s="4"/>
       <c r="F78" s="4"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="11" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>105</v>
+        <v>241</v>
       </c>
       <c r="D79" s="11" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="E79" s="4"/>
       <c r="F79" s="4"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A80" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="C80" t="s">
-        <v>118</v>
+      <c r="A80" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B80" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>242</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>187</v>
-      </c>
-      <c r="F80" s="1"/>
+        <v>159</v>
+      </c>
+      <c r="E80" s="4"/>
+      <c r="F80" s="4"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="B81" s="4" t="s">
-        <v>120</v>
+        <v>245</v>
+      </c>
+      <c r="B81" s="13" t="s">
+        <v>246</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>121</v>
+        <v>247</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>186</v>
+        <v>213</v>
       </c>
       <c r="E81" s="4"/>
-      <c r="F81" s="4"/>
+      <c r="F81" s="4" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A82" s="6">
-        <v>69</v>
-      </c>
-      <c r="B82" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="C82" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="D82" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="F82" t="s">
-        <v>173</v>
-      </c>
+      <c r="A82" s="11"/>
+      <c r="B82" s="13"/>
+      <c r="C82" s="4"/>
+      <c r="D82" s="11"/>
+      <c r="E82" s="4"/>
+      <c r="F82" s="4"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A83" s="6">
-        <v>70</v>
+      <c r="A83" s="6" t="s">
+        <v>101</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="C83" s="4" t="s">
-        <v>124</v>
+        <v>102</v>
+      </c>
+      <c r="C83" t="s">
+        <v>243</v>
       </c>
       <c r="D83" s="11" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F83" s="1"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A84" s="6">
-        <v>71</v>
+      <c r="A84" s="11" t="s">
+        <v>103</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>125</v>
+        <v>104</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>126</v>
+        <v>244</v>
       </c>
       <c r="D84" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="F84" s="1"/>
+        <v>159</v>
+      </c>
+      <c r="E84" s="4"/>
+      <c r="F84" s="4"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" s="6">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="D85" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="E85" s="1"/>
-      <c r="F85" s="4" t="s">
-        <v>115</v>
+        <v>144</v>
+      </c>
+      <c r="D85" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="F85" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="6">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>130</v>
+        <v>107</v>
       </c>
       <c r="D86" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="E86" s="1"/>
-      <c r="F86" s="4" t="s">
-        <v>115</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="F86" s="1"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="6">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>131</v>
+        <v>108</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
       <c r="D87" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="F87" t="s">
-        <v>115</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="F87" s="1"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" s="6">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>133</v>
+        <v>110</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>134</v>
+        <v>112</v>
       </c>
       <c r="D88" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="F88" t="s">
-        <v>115</v>
+        <v>136</v>
+      </c>
+      <c r="E88" s="1"/>
+      <c r="F88" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" s="6">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>237</v>
+        <v>111</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>238</v>
+        <v>113</v>
       </c>
       <c r="D89" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="F89" t="s">
+        <v>136</v>
+      </c>
+      <c r="E89" s="1"/>
+      <c r="F89" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A90" s="6">
+        <v>74</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C90" s="4" t="s">
         <v>115</v>
+      </c>
+      <c r="D90" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="F90" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" s="6">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>136</v>
+        <v>117</v>
+      </c>
+      <c r="D91" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="F91" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" s="6">
-        <v>129</v>
+        <v>76</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>137</v>
+        <v>200</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D92" s="6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A93" s="6">
-        <v>130</v>
-      </c>
-      <c r="B93" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="C93" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="D93" s="6" t="s">
-        <v>157</v>
+        <v>201</v>
+      </c>
+      <c r="D92" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="F92" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A94" s="6">
+        <v>128</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" s="6">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>174</v>
+        <v>120</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>175</v>
+        <v>123</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>157</v>
+        <v>249</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="6">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>176</v>
+        <v>121</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>177</v>
+        <v>122</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" s="6">
-        <v>146</v>
-      </c>
-      <c r="B97" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C97" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="D97" s="6" t="s">
-        <v>157</v>
+        <v>249</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A98" s="6">
+        <v>144</v>
+      </c>
+      <c r="B98" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B98" s="4" t="s">
-        <v>181</v>
-      </c>
       <c r="C98" s="4" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A99" s="6">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>182</v>
+        <v>149</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>183</v>
+        <v>150</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A100" s="6">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>184</v>
+        <v>151</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B101" s="4"/>
-      <c r="C101" s="4"/>
+      <c r="A101" s="6">
+        <v>147</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D101" s="6" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A102" s="6">
+        <v>148</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D102" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A103" s="6">
+        <v>149</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D103" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B104" s="4"/>
+      <c r="C104" s="4"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A105" s="6">
         <v>255</v>
       </c>
-      <c r="B102" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="C102" s="4" t="s">
+      <c r="B105" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C105" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="D102" s="6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B103" s="1"/>
-      <c r="C103" s="4"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B105" s="10" t="s">
-        <v>149</v>
+      <c r="D105" s="6" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B106" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B107" t="s">
-        <v>168</v>
-      </c>
+      <c r="B106" s="1"/>
+      <c r="C106" s="4"/>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B108" t="s">
-        <v>169</v>
+        <v>219</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B109" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B110" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added register returning status of remote programming via fiber
CHECKSUM=0x18D7
Timing for DDR clock fails badly, together with timing of some registers in DigiInterface/DIGILINK_0/Lane0/RX_CLK
</commit_message>
<xml_diff>
--- a/DRAC_Registers_timingconstrained.xlsx
+++ b/DRAC_Registers_timingconstrained.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tecchio/Desktop/work_instructions/ROC Manuals/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tecchio/Desktop/work_instructions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE21BBA-36A2-BD46-BB7D-EB7020B6E4D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61FD5200-A6D9-804C-A563-B5625357A617}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1400" yWindow="760" windowWidth="20140" windowHeight="18020" xr2:uid="{8033228E-8299-4C41-92C5-FE54786B42FA}"/>
+    <workbookView xWindow="1400" yWindow="760" windowWidth="25240" windowHeight="18020" xr2:uid="{8033228E-8299-4C41-92C5-FE54786B42FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="323">
   <si>
     <t>address</t>
   </si>
@@ -800,10 +800,211 @@
     <t>(*) Enabled by DCS_DIGIRW_SEL via reg=6</t>
   </si>
   <si>
-    <t>Last updated: May 4, 2025</t>
-  </si>
-  <si>
     <t>in units of 12.5 ns (80 MHz clock)</t>
+  </si>
+  <si>
+    <t>Last updated: May 23, 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DCS_PROG_RETURN </t>
+  </si>
+  <si>
+    <t>Valid only when DCS_CMD_STATUS=0x8000</t>
+  </si>
+  <si>
+    <t>return status of  REMOTE PROGRAMMABLE funcions</t>
+  </si>
+  <si>
+    <t>TESTDCSNGL</t>
+  </si>
+  <si>
+    <t>TESTDCSBLK</t>
+  </si>
+  <si>
+    <t>READSPI</t>
+  </si>
+  <si>
+    <t>READBACKBLK</t>
+  </si>
+  <si>
+    <t>READDEVICE</t>
+  </si>
+  <si>
+    <t>TALKTOADC</t>
+  </si>
+  <si>
+    <t>FINDALIGN</t>
+  </si>
+  <si>
+    <t>TALKTODIGI</t>
+  </si>
+  <si>
+    <t>READDATA</t>
+  </si>
+  <si>
+    <t>PREAMPGAIN</t>
+  </si>
+  <si>
+    <t>PREAMPTHRESH</t>
+  </si>
+  <si>
+    <t>PULSERON</t>
+  </si>
+  <si>
+    <t>PULSEROFF</t>
+  </si>
+  <si>
+    <t>MEASURETHRESH</t>
+  </si>
+  <si>
+    <t>READRATES</t>
+  </si>
+  <si>
+    <t>READGITREV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READILP </t>
+  </si>
+  <si>
+    <t>GETKEY</t>
+  </si>
+  <si>
+    <t>WRITEPREAMP</t>
+  </si>
+  <si>
+    <t>WRITECALDAC</t>
+  </si>
+  <si>
+    <t>READPREAMP</t>
+  </si>
+  <si>
+    <t>INITBYFIBER</t>
+  </si>
+  <si>
+    <t>REMOTEPROG</t>
+  </si>
+  <si>
+    <t>DIAGDATA</t>
+  </si>
+  <si>
+    <t>READDR</t>
+  </si>
+  <si>
+    <t>256-511</t>
+  </si>
+  <si>
+    <t>Reserved for fiber commands to uProc</t>
+  </si>
+  <si>
+    <t>Single WR to register 256 of  value V and read back via Single RD from register 256 of value V</t>
+  </si>
+  <si>
+    <t>BLOCK read of counters from 0 to N-1 specified by a DCS WRITE to register 257 of value N</t>
+  </si>
+  <si>
+    <t>write and read back BLOCK_WRITE of N values via "rocUtil block_write -a 259 -c N"</t>
+  </si>
+  <si>
+    <t>execute with Single DCS_WRITE of any value (ignored) followed by DCS_BLOCK_READ of 36 ADCs values</t>
+  </si>
+  <si>
+    <t>fiber version of GETDEVICEID</t>
+  </si>
+  <si>
+    <t>fiber version of READMONADCS</t>
+  </si>
+  <si>
+    <t>execute with Single DCS_WRITE of any value (ignored) followed by DCS_BLOCK_READ of 52 ID values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fiber version of ADCRWCMDID </t>
+  </si>
+  <si>
+    <t>parameters passed via BLOCK_WRITE and results read via simple read</t>
+  </si>
+  <si>
+    <t>fiber version of DIGIRW</t>
+  </si>
+  <si>
+    <t>fiber version of AUTOBITSLIPCMDID</t>
+  </si>
+  <si>
+    <t>parameters passed via SINGLE or BLOCK_WRITE - Does only 1 iteration!!</t>
+  </si>
+  <si>
+    <t>fiber version of READDATACMDID</t>
+  </si>
+  <si>
+    <t>parameters passed via BLOCK_WRITE</t>
+  </si>
+  <si>
+    <t>fiber version of SETPREAMPGAIN</t>
+  </si>
+  <si>
+    <t>fiber version of SETPREAMPTHRESHOLD</t>
+  </si>
+  <si>
+    <t>fiber version of SETPULSERON</t>
+  </si>
+  <si>
+    <t>fiber version of SETPULSEROFF</t>
+  </si>
+  <si>
+    <t>parameters passed via Single DCS WRITE</t>
+  </si>
+  <si>
+    <t>fiber version of MEASURETHRESHOLDCMDID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fiber version of READRATESCMDID </t>
+  </si>
+  <si>
+    <t>fiber version of GETGITREV</t>
+  </si>
+  <si>
+    <t>execute with Single DCS_WRITE of any value (ignored) followed by DCS_BLOCK_READ of size returned by reg 129</t>
+  </si>
+  <si>
+    <t>execute with Single DCS_WRITE of any value (ignored) followed by DCS_BLOCK_READ of 4 values</t>
+  </si>
+  <si>
+    <t>fiber version of GETILP</t>
+  </si>
+  <si>
+    <t>fiber version of READKEY</t>
+  </si>
+  <si>
+    <t>execute with Single DCS_WRITE of any value (ignored) followed by DCS_BLOCK_READ of of 4 values</t>
+  </si>
+  <si>
+    <t>write all gain&amp;thresh via BLOCK_WRITE of 96x4 parameters (96xGain CAL, 96xGain HV, 96xThresh CAL, 96xThres</t>
+  </si>
+  <si>
+    <t>fiber version of SETCALDAC</t>
+  </si>
+  <si>
+    <t>execute with Single DCS_WRITE of channel number followed by DCS_BLOCK_READ of 4 or 384 gain/thresh values</t>
+  </si>
+  <si>
+    <t>fiber version of DUMPSETTINGS</t>
+  </si>
+  <si>
+    <t>execute with Single DCS_WRITE of any value (ignored) followed by DCS_BLOCK_READ of 2 cal/hv errors</t>
+  </si>
+  <si>
+    <t>fiber version of INITDIGIS</t>
+  </si>
+  <si>
+    <t>fiber version of IAPROC</t>
+  </si>
+  <si>
+    <t>execute with BLOCK WRITE of at least 5 parameters, with first parameter specifying the action to take</t>
+  </si>
+  <si>
+    <t>Block RD of assorted diagnostics, started by a single WR of any value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DCS_BLOCK_READ of 1 kB block of DDR memory from address offset specified by reg 33&amp;34 </t>
   </si>
 </sst>
 </file>
@@ -1235,7 +1436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{518204DB-35D9-1947-A6E3-732720EF0C47}">
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.1640625" style="6" bestFit="1" customWidth="1"/>
@@ -1251,7 +1452,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -1808,7 +2009,7 @@
         <v>252</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -2676,125 +2877,482 @@
         <v>249</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A98" s="6">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A97" s="6">
+        <v>132</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="F97" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A99" s="6">
         <v>144</v>
       </c>
-      <c r="B98" s="4" t="s">
+      <c r="B99" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="C98" s="4" t="s">
+      <c r="C99" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="D98" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A99" s="6">
+      <c r="D99" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A100" s="6">
         <v>145</v>
       </c>
-      <c r="B99" s="4" t="s">
+      <c r="B100" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="C99" s="4" t="s">
+      <c r="C100" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="D99" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A100" s="6">
+      <c r="D100" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A101" s="6">
         <v>146</v>
       </c>
-      <c r="B100" s="4" t="s">
+      <c r="B101" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="C100" s="4" t="s">
+      <c r="C101" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="D100" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A101" s="6">
+      <c r="D101" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A102" s="6">
         <v>147</v>
       </c>
-      <c r="B101" s="4" t="s">
+      <c r="B102" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C101" s="4" t="s">
+      <c r="C102" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="D101" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A102" s="6">
+      <c r="D102" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A103" s="6">
         <v>148</v>
       </c>
-      <c r="B102" s="4" t="s">
+      <c r="B103" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C102" s="4" t="s">
+      <c r="C103" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="D102" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A103" s="6">
+      <c r="D103" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A104" s="6">
         <v>149</v>
       </c>
-      <c r="B103" s="4" t="s">
+      <c r="B104" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="C103" s="4" t="s">
+      <c r="C104" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="D103" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B104" s="4"/>
-      <c r="C104" s="4"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A105" s="6">
+      <c r="D104" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B105" s="4"/>
+      <c r="C105" s="4"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A106" s="6">
         <v>255</v>
       </c>
-      <c r="B105" s="4" t="s">
+      <c r="B106" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="C105" s="4" t="s">
+      <c r="C106" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="D105" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B106" s="1"/>
-      <c r="C106" s="4"/>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B108" t="s">
+      <c r="D106" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B107" s="1"/>
+      <c r="C107" s="4"/>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B109" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B109" t="s">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B110" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B110" t="s">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B111" t="s">
         <v>143</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A113" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="B113" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A114" s="6">
+        <v>256</v>
+      </c>
+      <c r="B114" t="s">
+        <v>259</v>
+      </c>
+      <c r="C114" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A115" s="6">
+        <v>257</v>
+      </c>
+      <c r="B115" t="s">
+        <v>260</v>
+      </c>
+      <c r="C115" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A116" s="6">
+        <v>258</v>
+      </c>
+      <c r="B116" t="s">
+        <v>261</v>
+      </c>
+      <c r="C116" t="s">
+        <v>289</v>
+      </c>
+      <c r="F116" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A117" s="6">
+        <v>259</v>
+      </c>
+      <c r="B117" t="s">
+        <v>262</v>
+      </c>
+      <c r="C117" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A118" s="6">
+        <v>260</v>
+      </c>
+      <c r="B118" t="s">
+        <v>263</v>
+      </c>
+      <c r="C118" t="s">
+        <v>292</v>
+      </c>
+      <c r="F118" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A119" s="6">
+        <v>262</v>
+      </c>
+      <c r="B119" t="s">
+        <v>264</v>
+      </c>
+      <c r="C119" t="s">
+        <v>294</v>
+      </c>
+      <c r="F119" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A120" s="6">
+        <v>263</v>
+      </c>
+      <c r="B120" t="s">
+        <v>266</v>
+      </c>
+      <c r="C120" t="s">
+        <v>294</v>
+      </c>
+      <c r="F120" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A121" s="6">
+        <v>264</v>
+      </c>
+      <c r="B121" t="s">
+        <v>265</v>
+      </c>
+      <c r="C121" t="s">
+        <v>297</v>
+      </c>
+      <c r="F121" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A122" s="6">
+        <v>265</v>
+      </c>
+      <c r="B122" t="s">
+        <v>267</v>
+      </c>
+      <c r="C122" t="s">
+        <v>299</v>
+      </c>
+      <c r="F122" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A123" s="6">
+        <v>266</v>
+      </c>
+      <c r="B123" t="s">
+        <v>268</v>
+      </c>
+      <c r="C123" t="s">
+        <v>299</v>
+      </c>
+      <c r="F123" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A124" s="6">
+        <v>267</v>
+      </c>
+      <c r="B124" t="s">
+        <v>269</v>
+      </c>
+      <c r="C124" t="s">
+        <v>299</v>
+      </c>
+      <c r="F124" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A125" s="6">
+        <v>268</v>
+      </c>
+      <c r="B125" t="s">
+        <v>270</v>
+      </c>
+      <c r="C125" t="s">
+        <v>299</v>
+      </c>
+      <c r="F125" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A126" s="6">
+        <v>269</v>
+      </c>
+      <c r="B126" t="s">
+        <v>271</v>
+      </c>
+      <c r="C126" t="s">
+        <v>304</v>
+      </c>
+      <c r="F126" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A127" s="6">
+        <v>270</v>
+      </c>
+      <c r="B127" t="s">
+        <v>272</v>
+      </c>
+      <c r="C127" t="s">
+        <v>299</v>
+      </c>
+      <c r="F127" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A128" s="6">
+        <v>271</v>
+      </c>
+      <c r="B128" t="s">
+        <v>273</v>
+      </c>
+      <c r="C128" t="s">
+        <v>299</v>
+      </c>
+      <c r="F128" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A129" s="6">
+        <v>272</v>
+      </c>
+      <c r="B129" t="s">
+        <v>274</v>
+      </c>
+      <c r="C129" t="s">
+        <v>308</v>
+      </c>
+      <c r="F129" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A130" s="6">
+        <v>273</v>
+      </c>
+      <c r="B130" t="s">
+        <v>275</v>
+      </c>
+      <c r="C130" t="s">
+        <v>309</v>
+      </c>
+      <c r="F130" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A131" s="6">
+        <v>274</v>
+      </c>
+      <c r="B131" t="s">
+        <v>276</v>
+      </c>
+      <c r="C131" t="s">
+        <v>312</v>
+      </c>
+      <c r="F131" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A132" s="6">
+        <v>275</v>
+      </c>
+      <c r="B132" t="s">
+        <v>277</v>
+      </c>
+      <c r="C132" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A133" s="6">
+        <v>276</v>
+      </c>
+      <c r="B133" t="s">
+        <v>278</v>
+      </c>
+      <c r="C133" t="s">
+        <v>299</v>
+      </c>
+      <c r="F133" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A134" s="6">
+        <v>277</v>
+      </c>
+      <c r="B134" t="s">
+        <v>279</v>
+      </c>
+      <c r="C134" t="s">
+        <v>315</v>
+      </c>
+      <c r="F134" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A135" s="6">
+        <v>278</v>
+      </c>
+      <c r="B135" t="s">
+        <v>280</v>
+      </c>
+      <c r="C135" t="s">
+        <v>317</v>
+      </c>
+      <c r="F135" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A137" s="6">
+        <v>384</v>
+      </c>
+      <c r="B137" t="s">
+        <v>281</v>
+      </c>
+      <c r="C137" t="s">
+        <v>320</v>
+      </c>
+      <c r="F137" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A139" s="6">
+        <v>511</v>
+      </c>
+      <c r="B139" t="s">
+        <v>282</v>
+      </c>
+      <c r="C139" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A140" s="6">
+        <v>512</v>
+      </c>
+      <c r="B140" t="s">
+        <v>283</v>
+      </c>
+      <c r="C140" t="s">
+        <v>322</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CRCSUM 0x00F8, meet timing with high effort
Added register to RS485 RX input. Added data header STATUS bits for HB and DREQ tag inconsistencies.
</commit_message>
<xml_diff>
--- a/DRAC_Registers_timingconstrained.xlsx
+++ b/DRAC_Registers_timingconstrained.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tecchio/Desktop/work_instructions/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tecchio/Desktop/work_instructions/ROC Manuals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61FD5200-A6D9-804C-A563-B5625357A617}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A032E91-9544-A74F-82A0-55499EE0A216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1400" yWindow="760" windowWidth="25240" windowHeight="18020" xr2:uid="{8033228E-8299-4C41-92C5-FE54786B42FA}"/>
   </bookViews>
@@ -893,9 +893,6 @@
     <t>256-511</t>
   </si>
   <si>
-    <t>Reserved for fiber commands to uProc</t>
-  </si>
-  <si>
     <t>Single WR to register 256 of  value V and read back via Single RD from register 256 of value V</t>
   </si>
   <si>
@@ -1005,6 +1002,9 @@
   </si>
   <si>
     <t xml:space="preserve">DCS_BLOCK_READ of 1 kB block of DDR memory from address offset specified by reg 33&amp;34 </t>
+  </si>
+  <si>
+    <t>REGISTER reserved for fiber commands to uProc</t>
   </si>
 </sst>
 </file>
@@ -3019,8 +3019,8 @@
       <c r="A113" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="B113" t="s">
-        <v>285</v>
+      <c r="B113" s="5" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.2">
@@ -3031,7 +3031,7 @@
         <v>259</v>
       </c>
       <c r="C114" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.2">
@@ -3042,7 +3042,7 @@
         <v>260</v>
       </c>
       <c r="C115" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.2">
@@ -3053,10 +3053,10 @@
         <v>261</v>
       </c>
       <c r="C116" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F116" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.2">
@@ -3067,7 +3067,7 @@
         <v>262</v>
       </c>
       <c r="C117" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.2">
@@ -3078,10 +3078,10 @@
         <v>263</v>
       </c>
       <c r="C118" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F118" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.2">
@@ -3092,10 +3092,10 @@
         <v>264</v>
       </c>
       <c r="C119" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F119" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.2">
@@ -3106,10 +3106,10 @@
         <v>266</v>
       </c>
       <c r="C120" t="s">
+        <v>293</v>
+      </c>
+      <c r="F120" t="s">
         <v>294</v>
-      </c>
-      <c r="F120" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.2">
@@ -3120,10 +3120,10 @@
         <v>265</v>
       </c>
       <c r="C121" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F121" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.2">
@@ -3134,10 +3134,10 @@
         <v>267</v>
       </c>
       <c r="C122" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F122" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.2">
@@ -3148,10 +3148,10 @@
         <v>268</v>
       </c>
       <c r="C123" t="s">
+        <v>298</v>
+      </c>
+      <c r="F123" t="s">
         <v>299</v>
-      </c>
-      <c r="F123" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.2">
@@ -3162,10 +3162,10 @@
         <v>269</v>
       </c>
       <c r="C124" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F124" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.2">
@@ -3176,10 +3176,10 @@
         <v>270</v>
       </c>
       <c r="C125" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F125" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.2">
@@ -3190,10 +3190,10 @@
         <v>271</v>
       </c>
       <c r="C126" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F126" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.2">
@@ -3204,10 +3204,10 @@
         <v>272</v>
       </c>
       <c r="C127" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F127" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.2">
@@ -3218,10 +3218,10 @@
         <v>273</v>
       </c>
       <c r="C128" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F128" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.2">
@@ -3232,10 +3232,10 @@
         <v>274</v>
       </c>
       <c r="C129" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F129" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.2">
@@ -3246,10 +3246,10 @@
         <v>275</v>
       </c>
       <c r="C130" t="s">
+        <v>308</v>
+      </c>
+      <c r="F130" t="s">
         <v>309</v>
-      </c>
-      <c r="F130" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.2">
@@ -3260,10 +3260,10 @@
         <v>276</v>
       </c>
       <c r="C131" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F131" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.2">
@@ -3274,7 +3274,7 @@
         <v>277</v>
       </c>
       <c r="C132" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.2">
@@ -3285,10 +3285,10 @@
         <v>278</v>
       </c>
       <c r="C133" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F133" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.2">
@@ -3299,10 +3299,10 @@
         <v>279</v>
       </c>
       <c r="C134" t="s">
+        <v>314</v>
+      </c>
+      <c r="F134" t="s">
         <v>315</v>
-      </c>
-      <c r="F134" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.2">
@@ -3313,10 +3313,10 @@
         <v>280</v>
       </c>
       <c r="C135" t="s">
+        <v>316</v>
+      </c>
+      <c r="F135" t="s">
         <v>317</v>
-      </c>
-      <c r="F135" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.2">
@@ -3327,10 +3327,10 @@
         <v>281</v>
       </c>
       <c r="C137" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F137" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.2">
@@ -3341,7 +3341,7 @@
         <v>282</v>
       </c>
       <c r="C139" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.2">
@@ -3352,7 +3352,7 @@
         <v>283</v>
       </c>
       <c r="C140" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remove NEWSPILL, add uProc interrupt and fix PREFETCH logic
See "commands_for_ROC_FW_timingconstrained.docx" for detailed about the firmware changes
</commit_message>
<xml_diff>
--- a/DRAC_Registers_timingconstrained.xlsx
+++ b/DRAC_Registers_timingconstrained.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tecchio/Desktop/work_instructions/ROC Manuals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A032E91-9544-A74F-82A0-55499EE0A216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9D65C0-6E6C-464B-A6F7-44D7EA6ED5E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1400" yWindow="760" windowWidth="25240" windowHeight="18020" xr2:uid="{8033228E-8299-4C41-92C5-FE54786B42FA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="333">
   <si>
     <t>address</t>
   </si>
@@ -122,9 +122,6 @@
     <t>Function</t>
   </si>
   <si>
-    <t>Event Marker delay in units of 5 ns ascalculated from loop back</t>
-  </si>
-  <si>
     <t>See bit-by-bit explanation below:</t>
   </si>
   <si>
@@ -554,9 +551,6 @@
     <t>If 1, set TWI control from uProc to fiber</t>
   </si>
   <si>
-    <t>If 1, run can be halted and counters/patterns are not reset after a null HB</t>
-  </si>
-  <si>
     <t>If 1, blinking sync fiber LED on key is turned off. If 0, LED is ON</t>
   </si>
   <si>
@@ -1005,6 +999,42 @@
   </si>
   <si>
     <t>REGISTER reserved for fiber commands to uProc</t>
+  </si>
+  <si>
+    <t>Event Marker delay in units of 5 ns as calculated from loop back</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If 1, run can be halted and counters/patterns are not reset after a null HB </t>
+  </si>
+  <si>
+    <t>Disabled in the firmware</t>
+  </si>
+  <si>
+    <t>DCS_EXT_SYS_IRQ0</t>
+  </si>
+  <si>
+    <t>If 1, it drives uProc IRQ0 for one 50MHz clock</t>
+  </si>
+  <si>
+    <t>bit(0)</t>
+  </si>
+  <si>
+    <t>Disables in ROC_FW "timeconstrained" branch</t>
+  </si>
+  <si>
+    <t>DIGIACTION</t>
+  </si>
+  <si>
+    <t>DIGIPROG</t>
+  </si>
+  <si>
+    <t>DIGIDONE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">read if DIGI PROGRAMMING is done </t>
+  </si>
+  <si>
+    <t>fiber version of PROGRAMDIGI</t>
   </si>
 </sst>
 </file>
@@ -1436,7 +1466,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{518204DB-35D9-1947-A6E3-732720EF0C47}">
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:F144"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.1640625" style="6" bestFit="1" customWidth="1"/>
@@ -1447,12 +1477,12 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -1472,7 +1502,7 @@
         <v>26</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -1485,19 +1515,19 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C6" t="s">
+        <v>203</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="s">
         <v>202</v>
-      </c>
-      <c r="C6" t="s">
-        <v>205</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -1508,10 +1538,10 @@
         <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>321</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1522,16 +1552,16 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C8" t="s">
+        <v>162</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E8" t="s">
         <v>161</v>
-      </c>
-      <c r="C8" t="s">
-        <v>163</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="E8" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -1539,10 +1569,10 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D9" s="6">
         <v>0</v>
@@ -1556,13 +1586,13 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E10" t="s">
         <v>3</v>
@@ -1570,13 +1600,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B11" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -1584,10 +1614,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B12" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>14</v>
@@ -1598,7 +1628,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B13" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
         <v>24</v>
@@ -1612,7 +1642,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B14" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
         <v>16</v>
@@ -1626,7 +1656,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B15" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
         <v>17</v>
@@ -1640,7 +1670,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B16" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C16" t="s">
         <v>18</v>
@@ -1654,13 +1684,13 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B17" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="C17" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="C17" t="s">
-        <v>98</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -1668,13 +1698,13 @@
     </row>
     <row r="18" spans="1:6" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" t="s">
         <v>38</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>40</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -1682,16 +1712,19 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B19" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C19" t="s">
-        <v>172</v>
+        <v>322</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E19">
         <v>0</v>
+      </c>
+      <c r="F19" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -1699,10 +1732,10 @@
         <v>9</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C20" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D20" s="6">
         <v>0</v>
@@ -1711,7 +1744,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -1719,10 +1752,10 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C21" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D21" s="6">
         <v>0</v>
@@ -1731,7 +1764,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -1742,158 +1775,164 @@
         <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E22">
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="14">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="6">
+        <v>15</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="C23" t="s">
+        <v>325</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="14">
         <v>17</v>
       </c>
-      <c r="B23" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="C23" s="15" t="s">
-        <v>251</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="6">
-        <v>23</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="C24" t="s">
-        <v>177</v>
-      </c>
-      <c r="D24" s="6">
-        <v>0</v>
-      </c>
-      <c r="E24">
-        <v>0</v>
-      </c>
-      <c r="F24" t="s">
-        <v>45</v>
+      <c r="B24" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="E24" s="15">
+        <v>0</v>
+      </c>
+      <c r="F24" s="15" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="6">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C25" t="s">
-        <v>178</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>140</v>
+        <v>175</v>
+      </c>
+      <c r="D25" s="6">
+        <v>0</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
       <c r="F25" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C26" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E26">
         <v>0</v>
+      </c>
+      <c r="F26" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C27" t="s">
-        <v>180</v>
-      </c>
-      <c r="D27" s="6">
-        <v>0</v>
+        <v>177</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>135</v>
       </c>
       <c r="E27">
         <v>0</v>
-      </c>
-      <c r="F27" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C28" t="s">
-        <v>181</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>140</v>
+        <v>178</v>
+      </c>
+      <c r="D28" s="6">
+        <v>0</v>
       </c>
       <c r="E28">
         <v>0</v>
       </c>
       <c r="F28" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="6">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C29" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E29">
         <v>0</v>
+      </c>
+      <c r="F29" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="6">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>47</v>
+        <v>186</v>
       </c>
       <c r="C30" t="s">
-        <v>127</v>
+        <v>180</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -1901,156 +1940,156 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="6">
+        <v>29</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" t="s">
+        <v>126</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" s="6">
         <v>30</v>
       </c>
-      <c r="B31" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="C31" t="s">
-        <v>128</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="E31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" s="11">
-        <v>31</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="D32" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="E32" s="4">
-        <v>0</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>131</v>
+      <c r="B32" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="C32" t="s">
+        <v>127</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="11">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>189</v>
+        <v>128</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="D33" s="11">
-        <v>0</v>
+        <v>129</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>138</v>
       </c>
       <c r="E33" s="4">
         <v>0</v>
       </c>
-      <c r="F33" s="4"/>
+      <c r="F33" s="4" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="11">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="D34" s="11" t="s">
-        <v>136</v>
+        <v>188</v>
+      </c>
+      <c r="D34" s="11">
+        <v>0</v>
       </c>
       <c r="E34" s="4">
         <v>0</v>
       </c>
-      <c r="F34" s="4" t="s">
-        <v>193</v>
-      </c>
+      <c r="F34" s="4"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="11">
+        <v>33</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="E35" s="4">
+        <v>0</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" s="11">
         <v>34</v>
       </c>
-      <c r="B35" s="12" t="s">
+      <c r="B36" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="C36" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="C35" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="D35" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="E35" s="4">
-        <v>0</v>
-      </c>
-      <c r="F35" s="4"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="11" t="s">
+      <c r="D36" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="E36" s="4">
+        <v>0</v>
+      </c>
+      <c r="F36" s="4"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="B36" s="12" t="s">
-        <v>246</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="D36" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="E36" s="4" t="s">
+      <c r="D37" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="F37" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="F36" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B38" s="10" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B40" s="5" t="s">
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B39" s="10" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B41" s="5" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A41" s="6">
-        <v>0</v>
-      </c>
-      <c r="B41" t="s">
-        <v>5</v>
-      </c>
-      <c r="C41" t="s">
-        <v>48</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="E41" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B42" t="s">
-        <v>202</v>
+        <v>5</v>
       </c>
       <c r="C42" t="s">
-        <v>206</v>
+        <v>47</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>207</v>
+        <v>135</v>
       </c>
       <c r="E42" t="s">
         <v>3</v>
@@ -2058,16 +2097,16 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B43" t="s">
-        <v>6</v>
+        <v>200</v>
       </c>
       <c r="C43" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>136</v>
+        <v>204</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>205</v>
       </c>
       <c r="E43" t="s">
         <v>3</v>
@@ -2075,16 +2114,16 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B44" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C44" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E44" t="s">
         <v>3</v>
@@ -2092,13 +2131,13 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C45" t="s">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>135</v>
@@ -2109,50 +2148,50 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B46" t="s">
-        <v>161</v>
+        <v>10</v>
       </c>
       <c r="C46" t="s">
-        <v>165</v>
+        <v>48</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="F46" t="s">
-        <v>166</v>
+        <v>134</v>
+      </c>
+      <c r="E46" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B47" t="s">
-        <v>11</v>
+        <v>160</v>
       </c>
       <c r="C47" t="s">
-        <v>50</v>
-      </c>
-      <c r="D47" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="E47" t="s">
-        <v>3</v>
+        <v>164</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="F47" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C48" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E48" t="s">
         <v>3</v>
@@ -2160,1199 +2199,1249 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B49" t="s">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="C49" t="s">
-        <v>99</v>
+        <v>13</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E49" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="6">
+        <v>8</v>
+      </c>
+      <c r="B50" t="s">
         <v>52</v>
       </c>
-      <c r="B50" t="s">
-        <v>54</v>
-      </c>
       <c r="C50" t="s">
-        <v>211</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="F50" s="3"/>
+        <v>98</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="E50" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B51" t="s">
+        <v>53</v>
+      </c>
+      <c r="C51" t="s">
+        <v>209</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="F51" s="3"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A52" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" t="s">
         <v>55</v>
       </c>
-      <c r="B51" t="s">
-        <v>56</v>
-      </c>
-      <c r="C51" t="s">
-        <v>70</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="F51" s="2"/>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A52" s="6">
-        <v>13</v>
-      </c>
-      <c r="B52" t="s">
-        <v>57</v>
-      </c>
       <c r="C52" t="s">
-        <v>58</v>
-      </c>
-      <c r="D52" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="F52" t="s">
-        <v>100</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="F52" s="2"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="6">
+        <v>13</v>
+      </c>
+      <c r="B53" t="s">
+        <v>56</v>
+      </c>
+      <c r="C53" t="s">
+        <v>57</v>
+      </c>
+      <c r="D53" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="F53" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A54" s="6">
         <v>14</v>
       </c>
-      <c r="B53" t="s">
-        <v>170</v>
-      </c>
-      <c r="C53" t="s">
+      <c r="B54" t="s">
         <v>169</v>
       </c>
-      <c r="D53" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="F53" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A54" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
+        <v>168</v>
+      </c>
+      <c r="D54" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="F54" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A55" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="B55" t="s">
+        <v>208</v>
+      </c>
+      <c r="C55" t="s">
         <v>210</v>
       </c>
-      <c r="C54" t="s">
-        <v>212</v>
-      </c>
-      <c r="D54" s="11" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A55" s="14">
+      <c r="D55" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A56" s="14">
         <v>17</v>
       </c>
-      <c r="B55" s="15" t="s">
+      <c r="B56" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="C56" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A57" s="6">
+        <v>18</v>
+      </c>
+      <c r="B57" t="s">
         <v>59</v>
       </c>
-      <c r="C55" s="15" t="s">
-        <v>196</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A56" s="6">
-        <v>18</v>
-      </c>
-      <c r="B56" t="s">
-        <v>60</v>
-      </c>
-      <c r="C56" t="s">
-        <v>226</v>
-      </c>
-      <c r="D56" s="6" t="s">
+      <c r="C57" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B57" t="s">
-        <v>168</v>
-      </c>
-      <c r="C57" t="s">
-        <v>228</v>
-      </c>
       <c r="D57" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="F57" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
-        <v>61</v>
+        <v>167</v>
       </c>
       <c r="C58" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>133</v>
+        <v>136</v>
+      </c>
+      <c r="F58" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C59" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A61" s="6">
-        <v>20</v>
-      </c>
-      <c r="B61" t="s">
-        <v>197</v>
-      </c>
-      <c r="C61" t="s">
-        <v>231</v>
-      </c>
-      <c r="D61" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="F61" t="s">
-        <v>199</v>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B60" t="s">
+        <v>61</v>
+      </c>
+      <c r="C60" t="s">
+        <v>228</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="6">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B62" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C62" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
+      </c>
+      <c r="F62" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="6">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B63" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
       <c r="C63" t="s">
-        <v>218</v>
-      </c>
-      <c r="D63" s="11" t="s">
-        <v>136</v>
+        <v>220</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="6">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B64" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C64" t="s">
         <v>216</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>225</v>
-      </c>
-      <c r="F64" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="6">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B65" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="C65" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>136</v>
+        <v>223</v>
+      </c>
+      <c r="F65" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" s="6">
+        <v>25</v>
+      </c>
+      <c r="B66" t="s">
+        <v>218</v>
+      </c>
+      <c r="C66" t="s">
+        <v>219</v>
+      </c>
+      <c r="D66" s="11" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A67" s="6">
         <v>26</v>
       </c>
-      <c r="B66" t="s">
-        <v>227</v>
-      </c>
-      <c r="C66" t="s">
+      <c r="B67" t="s">
+        <v>225</v>
+      </c>
+      <c r="C67" t="s">
+        <v>221</v>
+      </c>
+      <c r="D67" s="11" t="s">
         <v>223</v>
       </c>
-      <c r="D66" s="11" t="s">
-        <v>225</v>
-      </c>
-      <c r="F66" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A67" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B67" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C67" t="s">
-        <v>71</v>
-      </c>
-      <c r="D67" s="6" t="s">
-        <v>160</v>
-      </c>
       <c r="F67" t="s">
-        <v>100</v>
+        <v>140</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="6" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C68" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F68" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C69" t="s">
-        <v>234</v>
+        <v>71</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F69" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C70" t="s">
-        <v>84</v>
+        <v>232</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F70" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B71" s="13" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C71" t="s">
-        <v>232</v>
+        <v>83</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F71" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A72" s="11" t="s">
+      <c r="A72" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B72" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="B72" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="C72" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="D72" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="E72" s="4"/>
-      <c r="F72" s="4" t="s">
-        <v>100</v>
+      <c r="C72" t="s">
+        <v>230</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="F72" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="11" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B73" s="13" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="D73" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E73" s="4"/>
       <c r="F73" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B74" s="13" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D74" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E74" s="4"/>
       <c r="F74" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B75" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B75" s="13" t="s">
-        <v>83</v>
-      </c>
       <c r="C75" s="4" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D75" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E75" s="4"/>
       <c r="F75" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="11" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D76" s="11" t="s">
         <v>159</v>
       </c>
       <c r="E76" s="4"/>
-      <c r="F76" s="4"/>
+      <c r="F76" s="4" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="11" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D77" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E77" s="4"/>
       <c r="F77" s="4"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D78" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E78" s="4"/>
       <c r="F78" s="4"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D79" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E79" s="4"/>
       <c r="F79" s="4"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E80" s="4"/>
       <c r="F80" s="4"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B81" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="D81" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="E81" s="4"/>
+      <c r="F81" s="4"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A82" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="B82" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="C82" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="B81" s="13" t="s">
+      <c r="D82" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="E82" s="4"/>
+      <c r="F82" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="C81" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="D81" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="E81" s="4"/>
-      <c r="F81" s="4" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A82" s="11"/>
-      <c r="B82" s="13"/>
-      <c r="C82" s="4"/>
-      <c r="D82" s="11"/>
-      <c r="E82" s="4"/>
-      <c r="F82" s="4"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A83" s="6" t="s">
+      <c r="A83" s="11"/>
+      <c r="B83" s="13"/>
+      <c r="C83" s="4"/>
+      <c r="D83" s="11"/>
+      <c r="E83" s="4"/>
+      <c r="F83" s="4"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A84" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B84" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B83" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="C83" t="s">
-        <v>243</v>
-      </c>
-      <c r="D83" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="F83" s="1"/>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A84" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B84" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C84" s="4" t="s">
-        <v>244</v>
+      <c r="C84" t="s">
+        <v>241</v>
       </c>
       <c r="D84" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="E84" s="4"/>
-      <c r="F84" s="4"/>
+      <c r="F84" s="1"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A85" s="6">
-        <v>69</v>
+      <c r="A85" s="11" t="s">
+        <v>102</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="D85" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="F85" t="s">
-        <v>146</v>
-      </c>
+        <v>242</v>
+      </c>
+      <c r="D85" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="E85" s="4"/>
+      <c r="F85" s="4"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="6">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D86" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="F86" s="1"/>
+        <v>143</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="F86" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="6">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D87" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F87" s="1"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" s="6">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D88" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="E88" s="1"/>
-      <c r="F88" s="4" t="s">
-        <v>100</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="F88" s="1"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" s="6">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B89" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C89" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C89" s="4" t="s">
-        <v>113</v>
-      </c>
       <c r="D89" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E89" s="1"/>
       <c r="F89" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" s="6">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D90" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="F90" t="s">
-        <v>100</v>
+        <v>135</v>
+      </c>
+      <c r="E90" s="1"/>
+      <c r="F90" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" s="6">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D91" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F91" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" s="6">
+        <v>75</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D92" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="F92" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A93" s="6">
         <v>76</v>
       </c>
-      <c r="B92" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="C92" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="D92" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="F92" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A94" s="6">
-        <v>128</v>
-      </c>
-      <c r="B94" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="C94" s="4" t="s">
-        <v>119</v>
+      <c r="B93" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="D93" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="F93" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" s="6">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="D95" s="6" t="s">
-        <v>249</v>
+        <v>118</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="6">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C96" s="4" t="s">
         <v>122</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" s="6">
+        <v>130</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A98" s="6">
         <v>132</v>
       </c>
-      <c r="B97" s="4" t="s">
+      <c r="B98" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="C98" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="C97" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="D97" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="F97" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A99" s="6">
-        <v>144</v>
-      </c>
-      <c r="B99" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="D99" s="6" t="s">
-        <v>136</v>
+      <c r="D98" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="F98" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="6">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" s="6">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" s="6">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" s="6">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" s="6">
+        <v>148</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D104" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A105" s="6">
         <v>149</v>
       </c>
-      <c r="B104" s="4" t="s">
+      <c r="B105" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C105" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="C104" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="D104" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B105" s="4"/>
-      <c r="C105" s="4"/>
+      <c r="D105" s="6" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A106" s="6">
+      <c r="B106" s="4"/>
+      <c r="C106" s="4"/>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A107" s="6">
         <v>255</v>
       </c>
-      <c r="B106" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="C106" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="D106" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B107" s="1"/>
-      <c r="C107" s="4"/>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B109" t="s">
-        <v>219</v>
-      </c>
+      <c r="B107" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="D107" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B108" s="1"/>
+      <c r="C108" s="4"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B110" t="s">
-        <v>142</v>
+        <v>217</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B111" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A113" s="6" t="s">
-        <v>284</v>
-      </c>
-      <c r="B113" s="5" t="s">
-        <v>322</v>
+        <v>141</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B112" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A114" s="6">
-        <v>256</v>
-      </c>
-      <c r="B114" t="s">
-        <v>259</v>
-      </c>
-      <c r="C114" t="s">
-        <v>285</v>
+      <c r="A114" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" s="6">
+        <v>256</v>
+      </c>
+      <c r="B115" t="s">
         <v>257</v>
       </c>
-      <c r="B115" t="s">
-        <v>260</v>
-      </c>
       <c r="C115" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" s="6">
+        <v>257</v>
+      </c>
+      <c r="B116" t="s">
         <v>258</v>
       </c>
-      <c r="B116" t="s">
-        <v>261</v>
-      </c>
       <c r="C116" t="s">
-        <v>288</v>
-      </c>
-      <c r="F116" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" s="6">
+        <v>258</v>
+      </c>
+      <c r="B117" t="s">
         <v>259</v>
       </c>
-      <c r="B117" t="s">
-        <v>262</v>
-      </c>
       <c r="C117" t="s">
-        <v>287</v>
+        <v>286</v>
+      </c>
+      <c r="F117" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" s="6">
+        <v>259</v>
+      </c>
+      <c r="B118" t="s">
         <v>260</v>
       </c>
-      <c r="B118" t="s">
-        <v>263</v>
-      </c>
       <c r="C118" t="s">
-        <v>291</v>
-      </c>
-      <c r="F118" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" s="6">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B119" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C119" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="F119" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" s="6">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B120" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="C120" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="F120" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" s="6">
+        <v>263</v>
+      </c>
+      <c r="B121" t="s">
         <v>264</v>
       </c>
-      <c r="B121" t="s">
-        <v>265</v>
-      </c>
       <c r="C121" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="F121" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" s="6">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B122" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="C122" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="F122" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" s="6">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B123" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C123" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F123" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" s="6">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B124" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C124" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F124" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" s="6">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B125" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C125" t="s">
+        <v>296</v>
+      </c>
+      <c r="F125" t="s">
         <v>298</v>
-      </c>
-      <c r="F125" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" s="6">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B126" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C126" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="F126" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" s="6">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B127" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C127" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F127" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" s="6">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B128" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C128" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F128" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" s="6">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B129" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C129" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="F129" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" s="6">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B130" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C130" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F130" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" s="6">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B131" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C131" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="F131" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" s="6">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B132" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C132" t="s">
-        <v>312</v>
+        <v>309</v>
+      </c>
+      <c r="F132" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" s="6">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B133" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C133" t="s">
-        <v>298</v>
-      </c>
-      <c r="F133" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" s="6">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B134" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C134" t="s">
-        <v>314</v>
+        <v>296</v>
       </c>
       <c r="F134" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" s="6">
+        <v>277</v>
+      </c>
+      <c r="B135" t="s">
+        <v>277</v>
+      </c>
+      <c r="C135" t="s">
+        <v>312</v>
+      </c>
+      <c r="F135" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A136" s="6">
         <v>278</v>
       </c>
-      <c r="B135" t="s">
-        <v>280</v>
-      </c>
-      <c r="C135" t="s">
+      <c r="B136" t="s">
+        <v>278</v>
+      </c>
+      <c r="C136" t="s">
+        <v>314</v>
+      </c>
+      <c r="F136" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A138" s="6">
+        <v>384</v>
+      </c>
+      <c r="B138" t="s">
+        <v>279</v>
+      </c>
+      <c r="C138" t="s">
+        <v>317</v>
+      </c>
+      <c r="F138" t="s">
         <v>316</v>
-      </c>
-      <c r="F135" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A137" s="6">
-        <v>384</v>
-      </c>
-      <c r="B137" t="s">
-        <v>281</v>
-      </c>
-      <c r="C137" t="s">
-        <v>319</v>
-      </c>
-      <c r="F137" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" s="6">
-        <v>511</v>
+        <v>385</v>
       </c>
       <c r="B139" t="s">
-        <v>282</v>
+        <v>328</v>
       </c>
       <c r="C139" t="s">
-        <v>320</v>
+        <v>317</v>
+      </c>
+      <c r="F139" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" s="6">
+        <v>386</v>
+      </c>
+      <c r="B140" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A141" s="6">
+        <v>387</v>
+      </c>
+      <c r="B141" t="s">
+        <v>330</v>
+      </c>
+      <c r="C141" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A143" s="6">
+        <v>511</v>
+      </c>
+      <c r="B143" t="s">
+        <v>280</v>
+      </c>
+      <c r="C143" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A144" s="6">
         <v>512</v>
       </c>
-      <c r="B140" t="s">
-        <v>283</v>
-      </c>
-      <c r="C140" t="s">
-        <v>321</v>
+      <c r="B144" t="s">
+        <v>281</v>
+      </c>
+      <c r="C144" t="s">
+        <v>319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>